<commit_message>
update `UniteD-SRL - run span.xlsx`
</commit_message>
<xml_diff>
--- a/results/UniteD-SRL - run span.xlsx
+++ b/results/UniteD-SRL - run span.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e3f7d4e32ee84dc4/UniVe/UniteD-SRL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\vito\SRL\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="132" documentId="11_1EEB9EAE655331664673AAE434FE8CC552D62E15" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44E1FD46-0635-49FB-8E65-18A2FF85D402}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C701CD-63B3-490A-82B0-72128B197DB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41895" yWindow="1365" windowWidth="22965" windowHeight="15045" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-75" yWindow="10440" windowWidth="38580" windowHeight="10545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dependency-based" sheetId="1" r:id="rId1"/>
@@ -1103,53 +1103,53 @@
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="6">
-        <v>84.34</v>
+        <v>85.5</v>
       </c>
       <c r="J10" s="6">
-        <v>73.75</v>
+        <v>76.510000000000005</v>
       </c>
       <c r="K10" s="7">
-        <v>78.69</v>
+        <v>80.760000000000005</v>
       </c>
       <c r="L10" s="6"/>
       <c r="M10" s="6">
-        <v>37.47</v>
+        <v>37.54</v>
       </c>
       <c r="N10" s="6">
-        <v>2</v>
+        <v>3.58</v>
       </c>
       <c r="O10" s="7">
-        <v>3.8</v>
+        <v>6.53</v>
       </c>
       <c r="Q10" s="6">
-        <v>66.73</v>
+        <v>59.82</v>
       </c>
       <c r="R10" s="6">
-        <v>47.64</v>
+        <v>43.85</v>
       </c>
       <c r="S10" s="7">
-        <v>55.59</v>
+        <v>50.6</v>
       </c>
       <c r="U10" s="6">
-        <v>58.49</v>
+        <v>53.22</v>
       </c>
       <c r="V10" s="6">
-        <v>18.57</v>
+        <v>17.920000000000002</v>
       </c>
       <c r="W10" s="7">
-        <v>28.19</v>
+        <v>26.81</v>
       </c>
       <c r="Y10" s="6">
         <f>AVERAGE(I10,M10,Q10,U10)</f>
-        <v>61.757500000000007</v>
+        <v>59.019999999999996</v>
       </c>
       <c r="Z10" s="6">
         <f>AVERAGE(J10,N10,R10,V10)</f>
-        <v>35.49</v>
+        <v>35.465000000000003</v>
       </c>
       <c r="AA10" s="7">
         <f>AVERAGE(K10,O10,S10,W10)</f>
-        <v>41.567499999999995</v>
+        <v>41.175000000000004</v>
       </c>
       <c r="AB10" s="6"/>
       <c r="AC10" s="6"/>
@@ -1190,52 +1190,52 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>48.65</v>
+        <v>51.29</v>
       </c>
       <c r="J11">
-        <v>15.56</v>
+        <v>17.059999999999999</v>
       </c>
       <c r="K11" s="11">
-        <v>23.58</v>
+        <v>25.61</v>
       </c>
       <c r="M11">
-        <v>82.27</v>
+        <v>82.84</v>
       </c>
       <c r="N11">
-        <v>55.89</v>
+        <v>59.65</v>
       </c>
       <c r="O11" s="11">
-        <v>66.56</v>
+        <v>69.36</v>
       </c>
       <c r="Q11">
-        <v>44.17</v>
+        <v>50.13</v>
       </c>
       <c r="R11">
-        <v>14.42</v>
+        <v>16.559999999999999</v>
       </c>
       <c r="S11">
-        <v>21.74</v>
+        <v>24.9</v>
       </c>
       <c r="U11">
-        <v>29.99</v>
+        <v>41.31</v>
       </c>
       <c r="V11">
-        <v>6.3</v>
+        <v>9.69</v>
       </c>
       <c r="W11" s="11">
-        <v>10.41</v>
+        <v>15.7</v>
       </c>
       <c r="Y11" s="6">
         <f t="shared" ref="Y11:Y17" si="3">AVERAGE(I11,M11,Q11,U11)</f>
-        <v>51.269999999999996</v>
+        <v>56.392499999999998</v>
       </c>
       <c r="Z11" s="6">
         <f t="shared" ref="Z11:Z17" si="4">AVERAGE(J11,N11,R11,V11)</f>
-        <v>23.0425</v>
+        <v>25.74</v>
       </c>
       <c r="AA11" s="7">
         <f t="shared" ref="AA11:AA17" si="5">AVERAGE(K11,O11,S11,W11)</f>
-        <v>30.572499999999998</v>
+        <v>33.892499999999998</v>
       </c>
     </row>
     <row r="12" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1258,21 +1258,53 @@
       <c r="G12" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="K12" s="11"/>
-      <c r="O12" s="11"/>
-      <c r="S12" s="11"/>
-      <c r="W12" s="11"/>
-      <c r="Y12" s="6" t="e">
+      <c r="I12">
+        <v>86.34</v>
+      </c>
+      <c r="J12">
+        <v>77.760000000000005</v>
+      </c>
+      <c r="K12" s="11">
+        <v>81.819999999999993</v>
+      </c>
+      <c r="M12">
+        <v>82.81</v>
+      </c>
+      <c r="N12">
+        <v>60.1</v>
+      </c>
+      <c r="O12" s="11">
+        <v>69.650000000000006</v>
+      </c>
+      <c r="Q12">
+        <v>69.11</v>
+      </c>
+      <c r="R12">
+        <v>55.95</v>
+      </c>
+      <c r="S12" s="11">
+        <v>61.84</v>
+      </c>
+      <c r="U12">
+        <v>61.21</v>
+      </c>
+      <c r="V12">
+        <v>23.24</v>
+      </c>
+      <c r="W12" s="11">
+        <v>33.69</v>
+      </c>
+      <c r="Y12" s="6">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z12" s="6" t="e">
+        <v>74.867499999999993</v>
+      </c>
+      <c r="Z12" s="6">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA12" s="7" t="e">
+        <v>54.262500000000003</v>
+      </c>
+      <c r="AA12" s="7">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>61.75</v>
       </c>
     </row>
     <row r="13" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1295,21 +1327,53 @@
       <c r="G13" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="K13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="S13" s="11"/>
-      <c r="W13" s="11"/>
-      <c r="Y13" s="6" t="e">
+      <c r="I13" s="6">
+        <v>86.48</v>
+      </c>
+      <c r="J13" s="6">
+        <v>77.95</v>
+      </c>
+      <c r="K13" s="11">
+        <v>81.99</v>
+      </c>
+      <c r="M13" s="6">
+        <v>82.65</v>
+      </c>
+      <c r="N13" s="6">
+        <v>60.12</v>
+      </c>
+      <c r="O13" s="11">
+        <v>69.599999999999994</v>
+      </c>
+      <c r="Q13" s="6">
+        <v>77.16</v>
+      </c>
+      <c r="R13" s="6">
+        <v>71.78</v>
+      </c>
+      <c r="S13" s="11">
+        <v>74.37</v>
+      </c>
+      <c r="U13" s="6">
+        <v>60.89</v>
+      </c>
+      <c r="V13" s="6">
+        <v>23.1</v>
+      </c>
+      <c r="W13" s="11">
+        <v>33.5</v>
+      </c>
+      <c r="Y13" s="6">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z13" s="6" t="e">
+        <v>76.795000000000002</v>
+      </c>
+      <c r="Z13" s="6">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA13" s="7" t="e">
+        <v>58.237499999999997</v>
+      </c>
+      <c r="AA13" s="7">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>64.864999999999995</v>
       </c>
     </row>
     <row r="14" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1332,21 +1396,53 @@
       <c r="G14" s="15" t="b">
         <v>1</v>
       </c>
-      <c r="K14" s="11"/>
-      <c r="O14" s="11"/>
-      <c r="S14" s="11"/>
-      <c r="W14" s="11"/>
-      <c r="Y14" s="6" t="e">
+      <c r="I14" s="6">
+        <v>86.16</v>
+      </c>
+      <c r="J14" s="6">
+        <v>76.94</v>
+      </c>
+      <c r="K14" s="11">
+        <v>81.290000000000006</v>
+      </c>
+      <c r="M14" s="6">
+        <v>81.33</v>
+      </c>
+      <c r="N14" s="6">
+        <v>58.09</v>
+      </c>
+      <c r="O14" s="11">
+        <v>67.77</v>
+      </c>
+      <c r="Q14" s="6">
+        <v>70.06</v>
+      </c>
+      <c r="R14" s="6">
+        <v>45.86</v>
+      </c>
+      <c r="S14" s="11">
+        <v>55.43</v>
+      </c>
+      <c r="U14" s="6">
+        <v>75.52</v>
+      </c>
+      <c r="V14" s="6">
+        <v>63.68</v>
+      </c>
+      <c r="W14" s="11">
+        <v>69.099999999999994</v>
+      </c>
+      <c r="Y14" s="6">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Z14" s="6" t="e">
+        <v>78.267499999999998</v>
+      </c>
+      <c r="Z14" s="6">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA14" s="7" t="e">
+        <v>61.142499999999998</v>
+      </c>
+      <c r="AA14" s="7">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>68.397500000000008</v>
       </c>
     </row>
     <row r="15" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4244,6 +4340,13 @@
     <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="Y2:AA2"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="M2:O2"/>
+    <mergeCell ref="U2:W2"/>
     <mergeCell ref="AF17:AK17"/>
     <mergeCell ref="AM17:AR17"/>
     <mergeCell ref="I1:K1"/>
@@ -4251,13 +4354,6 @@
     <mergeCell ref="U1:W1"/>
     <mergeCell ref="Y1:AA1"/>
     <mergeCell ref="M1:O1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="Y2:AA2"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="M2:O2"/>
-    <mergeCell ref="U2:W2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Span EN and ZH result files updated
</commit_message>
<xml_diff>
--- a/results/UniteD-SRL - run span.xlsx
+++ b/results/UniteD-SRL - run span.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lorpa\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lorpa\Documents\Università\Magistrale\Anno2\TESI\project\SRL\SRL\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{877721C0-D82D-4926-83E9-AA1F1CD42559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D717C43D-C8C1-4378-99EC-2C6BBA294CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -710,53 +710,53 @@
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="6">
-        <v>1.68</v>
+        <v>61.11</v>
       </c>
       <c r="J4" s="6">
-        <v>22.05</v>
+        <v>12.9</v>
       </c>
       <c r="K4" s="7">
-        <v>0</v>
+        <v>21.3</v>
       </c>
       <c r="L4" s="6"/>
       <c r="M4" s="6">
-        <v>2.38</v>
+        <v>37.08</v>
       </c>
       <c r="N4" s="6">
-        <v>25.17</v>
+        <v>0.25</v>
       </c>
       <c r="O4" s="7">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q4" s="6">
-        <v>6.68</v>
+        <v>50.39</v>
       </c>
       <c r="R4" s="6">
-        <v>42.32</v>
+        <v>5.4</v>
       </c>
       <c r="S4" s="7">
-        <v>0</v>
+        <v>9.7899999999999991</v>
       </c>
       <c r="U4" s="6">
-        <v>8.1199999999999992</v>
+        <v>56.5</v>
       </c>
       <c r="V4" s="6">
-        <v>45.74</v>
+        <v>3.97</v>
       </c>
       <c r="W4" s="7">
-        <v>0</v>
+        <v>7.42</v>
       </c>
       <c r="Y4" s="6">
         <f t="shared" ref="Y4:Y9" si="0">AVERAGE(I4,M4,Q4,U4)</f>
-        <v>4.7149999999999999</v>
+        <v>51.269999999999996</v>
       </c>
       <c r="Z4" s="6">
         <f t="shared" ref="Z4:Z9" si="1">AVERAGE(J4,N4,R4,V4)</f>
-        <v>33.82</v>
+        <v>5.63</v>
       </c>
       <c r="AA4" s="7">
         <f t="shared" ref="AA4:AA9" si="2">AVERAGE(K4,O4,S4,W4)</f>
-        <v>0</v>
+        <v>9.7524999999999995</v>
       </c>
       <c r="AB4" s="6"/>
       <c r="AC4" s="6"/>
@@ -798,53 +798,53 @@
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="6">
-        <v>1.38</v>
+        <v>33.21</v>
       </c>
       <c r="J5" s="6">
-        <v>15.05</v>
+        <v>1.7</v>
       </c>
       <c r="K5" s="7">
-        <v>0</v>
+        <v>3.24</v>
       </c>
       <c r="L5" s="6"/>
       <c r="M5" s="6">
-        <v>1.78</v>
+        <v>51.65</v>
       </c>
       <c r="N5" s="6">
-        <v>14.94</v>
+        <v>8.9499999999999993</v>
       </c>
       <c r="O5" s="7">
-        <v>0</v>
+        <v>15.26</v>
       </c>
       <c r="Q5" s="6">
-        <v>1.06</v>
+        <v>28.21</v>
       </c>
       <c r="R5" s="6">
-        <v>14.78</v>
+        <v>0.64</v>
       </c>
       <c r="S5" s="7">
-        <v>0</v>
+        <v>1.25</v>
       </c>
       <c r="U5" s="6">
-        <v>0.89</v>
+        <v>33.76</v>
       </c>
       <c r="V5" s="6">
-        <v>14.73</v>
+        <v>0.74</v>
       </c>
       <c r="W5" s="7">
-        <v>0</v>
+        <v>1.46</v>
       </c>
       <c r="Y5" s="6">
         <f t="shared" si="0"/>
-        <v>1.2775000000000001</v>
+        <v>36.707499999999996</v>
       </c>
       <c r="Z5" s="6">
         <f t="shared" si="1"/>
-        <v>14.875</v>
+        <v>3.0074999999999998</v>
       </c>
       <c r="AA5" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.3025000000000002</v>
       </c>
       <c r="AB5" s="6"/>
       <c r="AC5" s="6"/>
@@ -4509,6 +4509,13 @@
     <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="AF17:AK17"/>
+    <mergeCell ref="AM17:AR17"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="U1:W1"/>
+    <mergeCell ref="Y1:AA1"/>
+    <mergeCell ref="M1:O1"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="I2:K2"/>
     <mergeCell ref="Q2:S2"/>
@@ -4516,13 +4523,6 @@
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="M2:O2"/>
     <mergeCell ref="U2:W2"/>
-    <mergeCell ref="AF17:AK17"/>
-    <mergeCell ref="AM17:AR17"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="U1:W1"/>
-    <mergeCell ref="Y1:AA1"/>
-    <mergeCell ref="M1:O1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>